<commit_message>
Add Doran to top comparison
</commit_message>
<xml_diff>
--- a/asian_games_lol_selection_data.xlsx
+++ b/asian_games_lol_selection_data.xlsx
@@ -30,11 +30,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'GOLGG_StageOnly_Check'!$A$1:$G$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Worlds_KeSPA'!$A$1:$I$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'AllPro'!$A$1:$G$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'POG_POM'!$A$1:$G$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'POG_POM'!$A$1:$G$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Validation_Report'!$A$1:$D$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Detailed_Stats_TODO'!$A$1:$D$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Weights'!$A$1:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Candidate_Summary'!$A$1:$J$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Candidate_Summary'!$A$1:$J$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1431,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1868,8 +1868,45 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Doran</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>55.56</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>56.52</v>
+      </c>
+      <c r="I12" s="2">
+        <f>B12*Weights!$B$2+C12*Weights!$B$3+D12*Weights!$B$4+F12*Weights!$B$5+H12*Weights!$B$6</f>
+        <v/>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Example only: default score maps; normalization is selected/contender scoped; not official.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J11"/>
+  <autoFilter ref="A1:J12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2843,12 +2880,12 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>context</t>
+          <t>contender</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>top/context</t>
+          <t>top</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -12167,7 +12204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -12295,19 +12332,19 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Canyon</t>
+          <t>Doran</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
@@ -12328,19 +12365,19 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Oner</t>
+          <t>Canyon</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -12361,7 +12398,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Faker</t>
+          <t>Oner</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -12370,10 +12407,10 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1100</v>
+        <v>600</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1100</v>
+        <v>600</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -12394,19 +12431,19 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Zeka</t>
+          <t>Faker</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -12427,19 +12464,19 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Gumayusi</t>
+          <t>Zeka</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>300</v>
+        <v>1000</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>300</v>
+        <v>1000</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -12460,19 +12497,19 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Peyz</t>
+          <t>Gumayusi</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
@@ -12493,19 +12530,19 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Viper</t>
+          <t>Peyz</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
@@ -12526,12 +12563,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Keria</t>
+          <t>Viper</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
@@ -12549,7 +12586,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2024 LCK Summer</t>
+          <t>2024 LCK Spring</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -12559,7 +12596,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Zeus</t>
+          <t>Keria</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -12568,14 +12605,14 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>S2</t>
         </is>
       </c>
     </row>
@@ -12592,12 +12629,12 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Kiin</t>
+          <t>Zeus</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
@@ -12625,7 +12662,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Canyon</t>
+          <t>Kiin</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -12634,10 +12671,10 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -12658,19 +12695,19 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Oner</t>
+          <t>Doran</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
@@ -12691,19 +12728,19 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Faker</t>
+          <t>Canyon</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
@@ -12724,19 +12761,19 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Zeka</t>
+          <t>Oner</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
@@ -12757,7 +12794,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Gumayusi</t>
+          <t>Faker</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -12766,10 +12803,10 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -12790,19 +12827,19 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Peyz</t>
+          <t>Zeka</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>1100</v>
+        <v>400</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>1100</v>
+        <v>400</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
@@ -12823,12 +12860,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Viper</t>
+          <t>Gumayusi</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
@@ -12856,19 +12893,19 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Keria</t>
+          <t>Peyz</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>400</v>
+        <v>1100</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>400</v>
+        <v>1100</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
@@ -12879,17 +12916,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2025 LCK Rounds 1-2</t>
+          <t>2024 LCK Summer</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>POM times</t>
+          <t>POG points</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Zeus</t>
+          <t>Viper</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -12898,47 +12935,47 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>7</v>
+        <v>400</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>700</v>
+        <v>400</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S3</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2025 LCK Rounds 1-2</t>
+          <t>2024 LCK Summer</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>POM times</t>
+          <t>POG points</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Kiin</t>
+          <t>Keria</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>2</v>
+        <v>400</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S3</t>
         </is>
       </c>
     </row>
@@ -12955,19 +12992,19 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Canyon</t>
+          <t>Zeus</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>100</v>
+        <v>700</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -12988,19 +13025,19 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Oner</t>
+          <t>Kiin</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
@@ -13021,7 +13058,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Faker</t>
+          <t>Doran</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -13030,10 +13067,10 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
@@ -13054,19 +13091,19 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Zeka</t>
+          <t>Canyon</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
@@ -13087,7 +13124,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Gumayusi</t>
+          <t>Oner</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -13096,10 +13133,10 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
@@ -13120,19 +13157,19 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Viper</t>
+          <t>Faker</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
@@ -13153,19 +13190,19 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Keria</t>
+          <t>Zeka</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -13176,7 +13213,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2025 LCK Rounds 3-5</t>
+          <t>2025 LCK Rounds 1-2</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -13186,12 +13223,12 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Zeus</t>
+          <t>Gumayusi</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
@@ -13202,14 +13239,14 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>S4</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2025 LCK Rounds 3-5</t>
+          <t>2025 LCK Rounds 1-2</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -13219,12 +13256,12 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Kiin</t>
+          <t>Viper</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
@@ -13235,14 +13272,14 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>S4</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2025 LCK Rounds 3-5</t>
+          <t>2025 LCK Rounds 1-2</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -13252,23 +13289,23 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Canyon</t>
+          <t>Keria</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>S4</t>
         </is>
       </c>
     </row>
@@ -13285,12 +13322,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Gumayusi</t>
+          <t>Zeus</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
@@ -13318,19 +13355,19 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Viper</t>
+          <t>Kiin</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
@@ -13351,7 +13388,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Keria</t>
+          <t>Doran</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -13360,10 +13397,10 @@
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
@@ -13384,7 +13421,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Ruler</t>
+          <t>Canyon</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -13393,10 +13430,10 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
@@ -13407,132 +13444,132 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2025 KeSPA Cup</t>
+          <t>2025 LCK Rounds 3-5</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>POG points</t>
+          <t>POM times</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Zeus</t>
+          <t>Gumayusi</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>S7</t>
+          <t>S5</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2025 KeSPA Cup</t>
+          <t>2025 LCK Rounds 3-5</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>POG points</t>
+          <t>POM times</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Oner</t>
+          <t>Viper</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>1</v>
+        <v>400</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>S7</t>
+          <t>S5</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2025 KeSPA Cup</t>
+          <t>2025 LCK Rounds 3-5</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>POG points</t>
+          <t>POM times</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Gumayusi</t>
+          <t>Keria</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>2</v>
+        <v>600</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>S7</t>
+          <t>S5</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2025 KeSPA Cup</t>
+          <t>2025 LCK Rounds 3-5</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>POG points</t>
+          <t>POM times</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Peyz</t>
+          <t>Ruler</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
         <v>4</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>4</v>
+        <v>400</v>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>S7</t>
+          <t>S5</t>
         </is>
       </c>
     </row>
@@ -13549,19 +13586,19 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Faker</t>
+          <t>Zeus</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
@@ -13582,7 +13619,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Keria</t>
+          <t>Doran</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -13591,10 +13628,10 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -13615,19 +13652,19 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Zeka</t>
+          <t>Oner</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
@@ -13638,17 +13675,17 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026 LCK Rounds 1-2 Snapshot</t>
+          <t>2025 KeSPA Cup</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>POM points</t>
+          <t>POG points</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Zeus</t>
+          <t>Gumayusi</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -13657,97 +13694,97 @@
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>200</v>
+        <v>2</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>200</v>
+        <v>2</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>S7</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026 LCK Rounds 1-2 Snapshot</t>
+          <t>2025 KeSPA Cup</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>POM points</t>
+          <t>POG points</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Kiin</t>
+          <t>Peyz</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>200</v>
+        <v>4</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>200</v>
+        <v>4</v>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>S7</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026 LCK Rounds 1-2 Snapshot</t>
+          <t>2025 KeSPA Cup</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>POM points</t>
+          <t>POG points</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Canyon</t>
+          <t>Faker</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>S7</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026 LCK Rounds 1-2 Snapshot</t>
+          <t>2025 KeSPA Cup</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>POM points</t>
+          <t>POG points</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Oner</t>
+          <t>Keria</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -13756,47 +13793,47 @@
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>300</v>
+        <v>5</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>300</v>
+        <v>5</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>S7</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2026 LCK Rounds 1-2 Snapshot</t>
+          <t>2025 KeSPA Cup</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>POM points</t>
+          <t>POG points</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Faker</t>
+          <t>Zeka</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>200</v>
+        <v>2</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>200</v>
+        <v>2</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>S7</t>
         </is>
       </c>
     </row>
@@ -13813,7 +13850,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Zeka</t>
+          <t>Zeus</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -13822,10 +13859,10 @@
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
@@ -13846,19 +13883,19 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Gumayusi</t>
+          <t>Kiin</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
@@ -13879,7 +13916,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Peyz</t>
+          <t>Doran</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -13912,19 +13949,19 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Keria</t>
+          <t>Canyon</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
@@ -13945,28 +13982,226 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
+          <t>Oner</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026 LCK Rounds 1-2 Snapshot</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>POM points</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Faker</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026 LCK Rounds 1-2 Snapshot</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>POM points</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Zeka</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>HLE</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026 LCK Rounds 1-2 Snapshot</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>POM points</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Gumayusi</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>HLE</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026 LCK Rounds 1-2 Snapshot</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>POM points</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Peyz</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026 LCK Rounds 1-2 Snapshot</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>POM points</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Keria</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026 LCK Rounds 1-2 Snapshot</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>POM points</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
           <t>Kanavi</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>HLE</t>
         </is>
       </c>
-      <c r="E54" s="2" t="n">
+      <c r="E60" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="F54" s="2" t="n">
+      <c r="F60" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G54"/>
+  <autoFilter ref="A1:G60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Ruler to bot comparison
</commit_message>
<xml_diff>
--- a/asian_games_lol_selection_data.xlsx
+++ b/asian_games_lol_selection_data.xlsx
@@ -23,18 +23,18 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$B$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$E$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$E$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Players'!$A$1:$F$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'League_Standings'!$A$1:$M$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'League_By_Player'!$A$1:$N$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'League_Standings'!$A$1:$M$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'League_By_Player'!$A$1:$N$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'GOLGG_StageOnly_Check'!$A$1:$G$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Worlds_KeSPA'!$A$1:$I$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'AllPro'!$A$1:$G$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'POG_POM'!$A$1:$G$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'AllPro'!$A$1:$G$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'POG_POM'!$A$1:$G$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Validation_Report'!$A$1:$D$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Detailed_Stats_TODO'!$A$1:$D$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Weights'!$A$1:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Candidate_Summary'!$A$1:$J$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Candidate_Summary'!$A$1:$J$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -734,12 +734,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Changed Viper/BLG 2026 Split 1 league row from playoff champion rank 1 to regular Group Ascend rank 2; added JDG/Peyz 2025 Split 1 regular row.</t>
+          <t>Changed Viper/BLG 2026 Split 1 league row from playoff champion rank 1 to regular Group Ascend rank 2; added JDG/Peyz 2025 Split 1 and JDG/Ruler 2024 Spring/Summer regular rows.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Do not run final Gumayusi-Peyz-Viper weighting until missing LPL Split 2/3 regular and POG/POM rows are completed.</t>
+          <t>Do not run final bot-lane weighting until missing Peyz/Viper LPL Split 2/3 regular and POG/POM rows are completed.</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>LPL POG/POM/MVP rows for Peyz and Viper are not collected in POG_POM.</t>
+          <t>Ruler 2024 LPL Man of the Match rows are collected; Peyz and Viper LPL POG/POM/MVP rows are still not collected in POG_POM.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1431,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1834,17 +1834,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Keria</t>
+          <t>Ruler</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>6</v>
@@ -1853,10 +1853,10 @@
         <v>66.67</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>2105</v>
+        <v>2200</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>91.52</v>
+        <v>95.65000000000001</v>
       </c>
       <c r="I11" s="2">
         <f>B11*Weights!$B$2+C11*Weights!$B$3+D11*Weights!$B$4+F11*Weights!$B$5+H11*Weights!$B$6</f>
@@ -1871,29 +1871,29 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Doran</t>
+          <t>Keria</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>77.5</v>
+        <v>100</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>100</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>55.56</v>
+        <v>66.67</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>1300</v>
+        <v>2105</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>56.52</v>
+        <v>91.52</v>
       </c>
       <c r="I12" s="2">
         <f>B12*Weights!$B$2+C12*Weights!$B$3+D12*Weights!$B$4+F12*Weights!$B$5+H12*Weights!$B$6</f>
@@ -1905,8 +1905,45 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Doran</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>55.56</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>56.52</v>
+      </c>
+      <c r="I13" s="2">
+        <f>B13*Weights!$B$2+C13*Weights!$B$3+D13*Weights!$B$4+F13*Weights!$B$5+H13*Weights!$B$6</f>
+        <v/>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Example only: default score maps; normalization is selected/contender scoped; not official.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J12"/>
+  <autoFilter ref="A1:J13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1917,7 +1954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2423,8 +2460,58 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>LPL 2024 Spring - Leaguepedia</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>https://lol.fandom.com/wiki/LPL/2024_Season/Spring_Season</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Ruler/JDG 2024 LPL Spring regular, All-Pro, Man of the Match</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>LPL 2024 Summer - Leaguepedia</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>https://lol.fandom.com/wiki/LPL/2024_Season/Summer_Season</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Ruler/JDG 2024 LPL Summer regular, All-Pro, Man of the Match</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Summer MoM row uses the Leaguepedia table that includes placement-stage stats.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E20"/>
+  <autoFilter ref="A1:E22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2816,17 +2903,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>context</t>
+          <t>contender</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>bot/context</t>
+          <t>bot</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2025-2026 Gen.G</t>
+          <t>2024 JDG; 2025-2026 Gen.G</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -3885,7 +3972,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2025 LPL Split 1 Regular</t>
+          <t>2024 LPL Spring Regular</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -3895,7 +3982,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>2025 Split 1</t>
+          <t>2024 Spring</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -3904,41 +3991,41 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="G17" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G17" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="H17" s="2" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>S9</t>
+          <t>S20</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>regular group-stage row only; Split 2/3 regular rows still missing</t>
+          <t>regular season row; JDG rank 3</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026 LPL Split 1</t>
+          <t>2024 LPL Summer Regular</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -3948,48 +4035,154 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>2026 Split 1</t>
+          <t>2024 Summer</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>BLG</t>
+          <t>JDG</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I18" s="2" t="n">
         <v>10</v>
       </c>
       <c r="J18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Group Ascend row after placements; JDG rank 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2025 LPL Split 1 Regular</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>LPL</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>2025 Split 1</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>JDG</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="K18" s="2" t="n">
+      <c r="K19" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>regular group-stage row only; Split 2/3 regular rows still missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026 LPL Split 1</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>LPL</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>2026 Split 1</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>BLG</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K20" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>S10</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>regular group-stage row; BLG later won playoffs per S19</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M18"/>
+  <autoFilter ref="A1:M20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4000,7 +4193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N73"/>
+  <dimension ref="A1:N75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -8154,7 +8347,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2025 LPL Split 1 Regular</t>
+          <t>2024 LPL Spring Regular</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -8164,12 +8357,12 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>2025 Split 1</t>
+          <t>2024 Spring</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Peyz</t>
+          <t>Ruler</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -8178,41 +8371,41 @@
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G72" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="H72" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H72" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="I72" s="2" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="L72" s="2" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>S9</t>
+          <t>S20</t>
         </is>
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>regular group-stage row only; Split 2/3 regular rows still missing</t>
+          <t>regular season row; JDG rank 3</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>2026 LPL Split 1</t>
+          <t>2024 LPL Summer Regular</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -8222,53 +8415,169 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>2026 Split 1</t>
+          <t>2024 Summer</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Viper</t>
+          <t>Ruler</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>BLG</t>
+          <t>JDG</t>
         </is>
       </c>
       <c r="F73" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H73" s="2" t="n">
         <v>4</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>10</v>
       </c>
       <c r="K73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>Group Ascend row after placements; JDG rank 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2025 LPL Split 1 Regular</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>LPL</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>2025 Split 1</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Peyz</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>JDG</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="J74" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K74" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="L73" s="2" t="n">
+      <c r="L74" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>regular group-stage row only; Split 2/3 regular rows still missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026 LPL Split 1</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>LPL</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>2026 Split 1</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Viper</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>BLG</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I75" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J75" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K75" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L75" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="M73" s="2" t="inlineStr">
+      <c r="M75" s="2" t="inlineStr">
         <is>
           <t>S10</t>
         </is>
       </c>
-      <c r="N73" s="2" t="inlineStr">
+      <c r="N75" s="2" t="inlineStr">
         <is>
           <t>regular group-stage row; BLG later won playoffs per S19</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N73"/>
+  <autoFilter ref="A1:N75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10790,7 +11099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -12096,12 +12405,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2025 LPL Split 1</t>
+          <t>2024 LPL Spring</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Peyz</t>
+          <t>Ruler</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -12115,26 +12424,26 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>S9</t>
+          <t>S20</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2025 LPL Split 2</t>
+          <t>2024 LPL Summer</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Peyz</t>
+          <t>Ruler</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -12148,52 +12457,118 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>S17</t>
+          <t>S21</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>2025 LPL Split 1</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Peyz</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>BOT</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>JDG</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2025 LPL Split 2</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Peyz</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>BOT</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>JDG</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
           <t>2026 LPL Split 1</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Viper</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>BOT</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>BLG</t>
         </is>
       </c>
-      <c r="E42" s="2" t="n">
+      <c r="E44" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F42" s="2" t="n">
+      <c r="F44" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>S10</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G42"/>
+  <autoFilter ref="A1:G44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12204,7 +12579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -12982,66 +13357,66 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2025 LCK Rounds 1-2</t>
+          <t>2024 LPL Spring</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>POM times</t>
+          <t>MVP times</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Zeus</t>
+          <t>Ruler</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>JDG</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S20</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2025 LCK Rounds 1-2</t>
+          <t>2024 LPL Summer</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>POM times</t>
+          <t>MVP times</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Kiin</t>
+          <t>Ruler</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>JDG</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S21</t>
         </is>
       </c>
     </row>
@@ -13058,19 +13433,19 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Doran</t>
+          <t>Zeus</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>100</v>
+        <v>700</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
@@ -13091,7 +13466,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Canyon</t>
+          <t>Kiin</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -13100,10 +13475,10 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
@@ -13124,7 +13499,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Oner</t>
+          <t>Doran</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -13133,10 +13508,10 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
@@ -13157,19 +13532,19 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Faker</t>
+          <t>Canyon</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
@@ -13190,19 +13565,19 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Zeka</t>
+          <t>Oner</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -13223,7 +13598,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Gumayusi</t>
+          <t>Faker</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -13232,10 +13607,10 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
@@ -13256,7 +13631,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Viper</t>
+          <t>Zeka</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -13289,7 +13664,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Keria</t>
+          <t>Gumayusi</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -13298,10 +13673,10 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
@@ -13312,7 +13687,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2025 LCK Rounds 3-5</t>
+          <t>2025 LCK Rounds 1-2</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -13322,30 +13697,30 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Zeus</t>
+          <t>Ruler</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>S4</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2025 LCK Rounds 3-5</t>
+          <t>2025 LCK Rounds 1-2</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -13355,12 +13730,12 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Kiin</t>
+          <t>Viper</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
@@ -13371,14 +13746,14 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>S4</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2025 LCK Rounds 3-5</t>
+          <t>2025 LCK Rounds 1-2</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -13388,7 +13763,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Doran</t>
+          <t>Keria</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -13404,7 +13779,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>S4</t>
         </is>
       </c>
     </row>
@@ -13421,12 +13796,12 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Canyon</t>
+          <t>Zeus</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
@@ -13454,19 +13829,19 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Gumayusi</t>
+          <t>Kiin</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
@@ -13487,19 +13862,19 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Viper</t>
+          <t>Doran</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
@@ -13520,19 +13895,19 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Keria</t>
+          <t>Canyon</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>600</v>
+        <v>100</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
@@ -13553,19 +13928,19 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Ruler</t>
+          <t>Gumayusi</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
@@ -13576,17 +13951,17 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2025 KeSPA Cup</t>
+          <t>2025 LCK Rounds 3-5</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>POG points</t>
+          <t>POM times</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Zeus</t>
+          <t>Viper</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -13595,31 +13970,31 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>3</v>
+        <v>400</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>S7</t>
+          <t>S5</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2025 KeSPA Cup</t>
+          <t>2025 LCK Rounds 3-5</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>POG points</t>
+          <t>POM times</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Doran</t>
+          <t>Keria</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -13628,47 +14003,47 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>S7</t>
+          <t>S5</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2025 KeSPA Cup</t>
+          <t>2025 LCK Rounds 3-5</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>POG points</t>
+          <t>POM times</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Oner</t>
+          <t>Ruler</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>1</v>
+        <v>400</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>S7</t>
+          <t>S5</t>
         </is>
       </c>
     </row>
@@ -13685,7 +14060,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Gumayusi</t>
+          <t>Zeus</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -13694,10 +14069,10 @@
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
@@ -13718,7 +14093,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Peyz</t>
+          <t>Doran</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -13727,10 +14102,10 @@
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
@@ -13751,7 +14126,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Faker</t>
+          <t>Oner</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -13760,10 +14135,10 @@
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
@@ -13784,19 +14159,19 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Keria</t>
+          <t>Gumayusi</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
@@ -13817,19 +14192,19 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Zeka</t>
+          <t>Peyz</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
@@ -13840,99 +14215,99 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026 LCK Rounds 1-2 Snapshot</t>
+          <t>2025 KeSPA Cup</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>POM points</t>
+          <t>POG points</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Zeus</t>
+          <t>Faker</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>S7</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2026 LCK Rounds 1-2 Snapshot</t>
+          <t>2025 KeSPA Cup</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>POM points</t>
+          <t>POG points</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Kiin</t>
+          <t>Keria</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>200</v>
+        <v>5</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>200</v>
+        <v>5</v>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>S7</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026 LCK Rounds 1-2 Snapshot</t>
+          <t>2025 KeSPA Cup</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>POM points</t>
+          <t>POG points</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Doran</t>
+          <t>Zeka</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>S7</t>
         </is>
       </c>
     </row>
@@ -13949,19 +14324,19 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Canyon</t>
+          <t>Zeus</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Gen.G</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
@@ -13982,19 +14357,19 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Oner</t>
+          <t>Kiin</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
@@ -14015,7 +14390,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Faker</t>
+          <t>Doran</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -14024,10 +14399,10 @@
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
@@ -14048,19 +14423,19 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Zeka</t>
+          <t>Canyon</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
@@ -14081,19 +14456,19 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Gumayusi</t>
+          <t>Oner</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>HLE</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
@@ -14114,7 +14489,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Peyz</t>
+          <t>Faker</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -14123,10 +14498,10 @@
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
@@ -14147,19 +14522,19 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Keria</t>
+          <t>Zeka</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>HLE</t>
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
@@ -14180,28 +14555,127 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
+          <t>Gumayusi</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>HLE</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026 LCK Rounds 1-2 Snapshot</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>POM points</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Peyz</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026 LCK Rounds 1-2 Snapshot</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>POM points</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Keria</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026 LCK Rounds 1-2 Snapshot</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>POM points</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
           <t>Kanavi</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>HLE</t>
         </is>
       </c>
-      <c r="E60" s="2" t="n">
+      <c r="E63" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="F60" s="2" t="n">
+      <c r="F63" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G60"/>
+  <autoFilter ref="A1:G63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>